<commit_message>
/SKOtracking: correct stale figures against live dashboards
Verified against TikTok, OpenAI and Meta just now:

- Meta campaign budget $250 → $150/day, ceiling recalculated
- Meta creative "2 of 12 built" → 8 built, 8 pending publish
- TikTok spend $1,442.31 → $1,450.02; refunded to $100 and delivering
  again, 2 ad groups active, 13 still not delivering
- OpenAI order_created 0 → 3; purchases land after the schema fix

T-02 retitled. The blocker was "order_created has received zero events";
that is fixed. The real problem is coverage: 220 checkout_started against
634 actual orders means the pixel sees about a third of checkouts and
almost none of the purchases. Downgraded from blocker to high, since it
no longer stops a launch, and reworded to describe what is actually wrong.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/sko-tracking.xlsx
+++ b/public/sko-tracking.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -164,9 +164,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -656,7 +653,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>checkout_started healthy at 188 events. order_created at 0, with 180 rejected for invalid properties — traced to unsupported fields inside contents[] items, since the schema permits only id, name, content_type, quantity, amount and currency there. Schema alignment has shipped and validated with accepted_events: 1, but a real purchase has not yet been observed. Identifier coverage remains 0% on both email and external ID.</t>
+          <t>checkout_started 220, order_created 3 — purchases are now landing after the schema fix. Identifier coverage still 0% on both email and external ID. 220 pixel checkouts against 634 real orders means the pixel is missing most of the funnel.</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1372,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Open — gates campaign launch</t>
+          <t>Open — no purchase observed on the Meta dataset yet</t>
         </is>
       </c>
     </row>
@@ -1385,9 +1382,9 @@
           <t>T-02</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>blocker</t>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -1397,22 +1394,22 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>OpenAI order_created has received zero events</t>
+          <t>OpenAI pixel undercounts the funnel</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>checkout_started received 188 events; order_created received 0, with 180 rejected for invalid properties. OpenAI's schema resolves the cause: type is required and must be "contents" for both events, and amount must be an integer in ISO 4217 minor units, so cents was already correct. The strict rule is on contents[] items, which may carry only id, name, content_type, quantity, amount and currency — any additional field fails validation.</t>
+          <t>order_created has gone 0 → 3 since the schema fix, so purchases now land. But 220 checkout_started against 634 real orders means the pixel sees roughly a third of checkouts and almost no purchases.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Fix shipped: browser pixel and server CAPI now map each event to its documented data type, contents[] items carry only permitted fields in minor units, and unsupported fields are stripped server-side. Validated with accepted_events: 1.</t>
+          <t>Find why most orders never fire the pixel — installed mid-week, or a checkout path that skips it.</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Fix shipped — verify order_created rises above 0 from a real confirmation page</t>
+          <t>Open — schema fixed, coverage is not</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1456,7 @@
           <t>T-04</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -1496,7 +1493,7 @@
           <t>T-05</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -1589,7 +1586,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>$250.00 / day (campaign budget)</t>
+          <t>$150.00 / day (campaign budget)</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1598,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>$437.50 max in a day · $1,750 max in a week</t>
+          <t>$262.50 max in a day · $1,050 max in a week</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1634,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Off — unpublished draft, $0 spent</t>
+          <t>Off — 8 ads pending publish, $0 spent</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1646,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2 of 12 built</t>
+          <t>8 built</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1668,7 @@
           <t>Verified</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>

</xml_diff>

<commit_message>
/SKOtracking: Aug 11-17 refresh — spend, pixel state, issues, top ads, scorecard
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/sko-tracking.xlsx
+++ b/public/sko-tracking.xlsx
@@ -665,7 +665,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2122473828697675</t>
+          <t>1023230300704427</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>unverified</t>
+          <t>degraded</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>ID now matches the dataset the ad account optimizes against. Earlier today the site was firing 2089922941789319 instead. Events Manager still shows no conversion events recorded — needs one test order to confirm Purchase lands.</t>
+          <t>New dataset live in production since midweek — full funnel firing (PageView 2.4K, ViewContent 468, AddToCart 109, Checkout 40, Purchase 11). Purchase event is gated on payment verification and fires on ~10% of orders; fix ticketed. CAPI still blocked on system-user token.</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Server copy dedupes on the same meta_event_id as Meta. Sharing one key across two platforms works, but means a change to the key breaks both at once.</t>
+          <t>Server copy dedupes on the same meta_event_id as Meta. Purchase event shares the same payment-verification gate as Meta — TikTok-attributed counts undercount for the same reason. Fix ticketed.</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Week of Aug 4 – Aug 10, 2026</t>
+          <t>Week of Aug 11 – Aug 17, 2026</t>
         </is>
       </c>
     </row>
@@ -920,8 +920,12 @@
           <t>Ad spend</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n"/>
-      <c r="C4" s="13" t="n"/>
+      <c r="B4" s="13" t="n">
+        <v>9706.190000000001</v>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>5500</v>
+      </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Sum of Meta + TikTok + OpenAI + Google Ads Manager spend for the week</t>
@@ -934,11 +938,15 @@
           <t>Revenue attributed to ads</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
+      <c r="B5" s="13" t="n">
+        <v>33549</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>21000</v>
+      </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Order table where attribution_source is a paid channel. Your own orders are business truth, not the platforms' self-reported numbers</t>
+          <t>TikTok platform-reported (order-table floor pending capture fix)</t>
         </is>
       </c>
     </row>
@@ -948,11 +956,15 @@
           <t>Blended ROAS</t>
         </is>
       </c>
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="15" t="n"/>
+      <c r="B6" s="15" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>3.4</v>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Derived: revenue attributed to ads ÷ ad spend</t>
+          <t>Platform revenue ÷ total spend (TikTok+Meta). 3.4× = 10%-margin floor</t>
         </is>
       </c>
     </row>
@@ -962,11 +974,13 @@
           <t>Orders from ads</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
+      <c r="B7" s="16" t="n">
+        <v>160</v>
+      </c>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>Order table, paid attribution_source, same window</t>
+          <t>154 TikTok-attributed + 6 Meta tracked (platform-reported)</t>
         </is>
       </c>
     </row>
@@ -976,7 +990,9 @@
           <t>UGC videos posted</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n"/>
+      <c r="B8" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="C8" s="16" t="n"/>
       <c r="D8" s="14" t="inlineStr">
         <is>
@@ -990,11 +1006,13 @@
           <t>UGC views</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n"/>
+      <c r="B9" s="16" t="n">
+        <v>312000</v>
+      </c>
       <c r="C9" s="16" t="n"/>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>Creator-reported or pulled from each post's native analytics</t>
+          <t>Paid impressions across Ethan-content placements, TikTok, Aug 9–17</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1022,9 @@
           <t>Revenue attributed to UGC</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n"/>
+      <c r="B10" s="13" t="n">
+        <v>16699</v>
+      </c>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="14" t="inlineStr">
         <is>
@@ -1022,7 +1042,7 @@
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Revenue attributed to UGC is only as exact as the identifier on the order. A unique discount code per creator is the single highest-leverage change here: it survives ad blockers, iOS, and dark social sharing, none of which a click ID does. Without per-creator codes, UGC revenue is an estimate no matter how the tracking is built.</t>
+          <t>Revenue attributed to UGC is platform-reported and only as exact as the identifier on the order. Purchase-event capture fix (ticketed) is the gate to trusting the floor. Per-creator codes remain the identifier that survives ad blockers, iOS, and dark social.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1088,20 +1108,100 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ethan UGC_vKCU0o8b</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1632.98</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>7556.44</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>4.63</v>
+      </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>No ad has delivered an impression yet.</t>
+          <t>Native creator video, 2.12% CTR, runs profitably in 3 pools — the account's workhorse</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>EYE_GIANT_9X16_15s</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>506.5</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>4006.51</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Low CTR, high intent — $267 baskets, ~$70 profit/order; dedicated ad group next week</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ethan ugc 2 + new videos</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2345.17</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>9142.4</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Ethan's new content works (5.93×/3.44×); logo/background treatments ran ~1.0× and get throttled</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>TheBOX</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>34.44</v>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>First tracked Meta conversions: 6 purchases, $5.74 CPA, 100% men 25–34 — converts in-feed without link clicks</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1352,27 +1452,27 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Meta · TikTok</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Meta Purchase never confirmed firing</t>
+          <t>Purchase event fires on ~10% of orders</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>The ad set optimizes for Purchase on 2122473828697675, and Events Manager reports no conversion events set up on that dataset. Until a purchase is observed landing, the campaign would spend against a model with no signal.</t>
+          <t>The purchase event is gated on a payment-verified timestamp that usually lands after the confirmation page renders. ~140 orders since Friday produced 11 pixel purchases. Every platform's reported conversions and every bid decision run on a 10% sample.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Events Manager → dataset → Test Events → enter skocompounds.com → place one real order → confirm Purchase arrives with a value.</t>
+          <t>Fire the purchase event on order creation, unconditionally, every payment path — server-side if a path skips the confirmation page. Ticket sent to Lovable; acceptance is one full day where pixel purchases ≈ admin orders.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Open — no purchase observed on the Meta dataset yet</t>
+          <t>Open — ticket sent, highest priority</t>
         </is>
       </c>
     </row>
@@ -1521,6 +1621,43 @@
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Open — no longer blocks the pixel, still an access risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>T-06</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Meta payment errors throttle delivery</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Both campaigns show Payment error · low budget used. The company card caps unsupervised spend, so charges fail until pushed manually; every stall stops delivery and resets pacing.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Onboard the replacement card. Until then, expect Meta results to under-read the creative.</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Open — card swap in progress</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1699,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>SKO | Sales | Prospecting | Aug 2026</t>
+          <t>END OF SUMMER 30 · New Sales Campaign</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1711,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>880814205101777</t>
+          <t>2033203383989191 (SKO Ad Account – Compliant)</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1723,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>$150.00 / day (campaign budget)</t>
+          <t>$150/day intended; payment errors capping actual delivery</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1735,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>$262.50 max in a day · $1,050 max in a week</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1747,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>US · Broad · 20-65 · Purchase</t>
+          <t>END OF SUMMER 30 · Last Chance Summer 30</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1759,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Sales · Maximize conversions · Purchase</t>
+          <t>Sales · Purchase on dataset 1023230300704427</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1771,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Off — 8 ads pending publish, $0 spent</t>
+          <t>Live since Aug 13 · $677.58 spent Aug 1–17 · Payment error flags on both campaigns</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1783,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>8 built</t>
+          <t>ETHAN UGC summer 30 · PUREST · GIANTWOMAN + AI IMAGE · TheBOX</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1795,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SUMMER30 — 30% off, no end date, cancelled manually</t>
+          <t>SUMMER30 still reaching paid traffic — being pulled from paid; codes burned into some creatives (AI-4, HighCostBau) need re-cuts</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1807,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>